<commit_message>
Complete Task 10: P/R/F1 metrics + PDF report; refresh GT to 20 FR docs
</commit_message>
<xml_diff>
--- a/docs/ground_truth.xlsx
+++ b/docs/ground_truth.xlsx
@@ -507,7 +507,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Real_MaterialCert_EN_NST_Inspection.pdf</t>
+          <t>Real_MaterialCert_FR_Larobinetterie_134822.pdf</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -517,12 +517,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>scanned</t>
+          <t>digital</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -532,39 +532,39 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>EXP1390198</t>
+          <t>134822</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Kuang Tai Metal Industrial Co. Ltd.</t>
+          <t>La Robinetterie (LRI-Sodime)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>AWS A5.9 ER316LSi</t>
+          <t>1.4307 / 304L</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>400 Kgs</t>
+          <t>38 mm (dimension)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2013-11-05</t>
+          <t>2019-05-23</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Inspection certificate EN 10204 3.1. Lot No. 13A31001. Customer: Watanabe Trading. Issued by Norsk Sveiseteknikk (NST).</t>
+          <t>Certificat de Réception 3.1 NF EN 10204. Heat number A1804323. Article 8185X.38 (TE SMS 38 INOX 304L).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Real_MaterialCert_FR_Larobinetterie_134822.pdf</t>
+          <t>Real_MaterialCert_FR_Antelis_Dillinger_32.pdf</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -589,39 +589,39 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>134822</t>
+          <t>59003730</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>La Robinetterie (LRI-Sodime)</t>
+          <t>AG der Dillinger Hüttenwerke</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>1.4307 / 304L</t>
+          <t>S355G10+N</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>38 mm (dimension)</t>
+          <t>15642 KG</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2019-05-23</t>
+          <t>2018-09-26</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Certificat de Réception 3.1 NF EN 10204. Heat number A1804323. Article 8185X.38 (TE SMS 38 INOX 304L). No piece-count on face of cert.</t>
+          <t>Certificat de Réception 3.2 EN 10204:2004. Customer: Antelis Leudelange. Heat 460073. Effective mass 15940 KG.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Real_MaterialCert_FR_Antelis_Dillinger_32.pdf</t>
+          <t>Real_MaterialCert_FR_Larobinetterie_160629.pdf</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -646,39 +646,39 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>59003730</t>
+          <t>736145</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>AG der Dillinger Hüttenwerke</t>
+          <t>SIDERINOX</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>S355G10+N</t>
+          <t>AISI 304/304L (EN 1.4301/1.4307)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>15642 KG</t>
+          <t>312 m</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2018-09-26</t>
+          <t>2024-06-26</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Certificat de Réception 3.2 EN 10204:2004. Customer: Antelis Leudelange. Heat 460073. Effective mass 15940 KG.</t>
+          <t>Certificat d'essai EN 10204 3.1. Tube rond inox Ø 40 x 1 mm recuit brossé EN 10357 TC2 soudé. Client: La Robinetterie Industrielle. 284 kg poids total. DDT N°2725 du 26.06.2024.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Real_MaterialCert_EN_Blackmer.pdf</t>
+          <t>Real_MaterialCert_FR_Dillinger_Antelis.pdf</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -698,36 +698,44 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>real_template</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
+          <t>real_filled</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>409707-001</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Blackmer (PSG Dover)</t>
+          <t>AG der Dillinger Hüttenwerke</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>EN 10204 3.1 reference</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
+          <t>S355K2+N</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>25434 KG</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2015-03-01</t>
+          <t>2015-11-26</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Blackmer Form 588 — reference/index of sample cert types (MC/MCM/MR/MPT/PMI/PTR). Not a filled certificate; no heat/project/quantity on page 1.</t>
+          <t>Certificat de Réception 3.1 EN 10204:2004 / ISO 10474:2013. Customer: Antelis Leudelange. Avis d'expédition 6048684. 9 tôles 20x3000x6000 mm. Heat 427181. Norme NF-EN10025-2:05.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_MaterialCert_EN_01.pdf</t>
+          <t>Real_MaterialCert_FR_Ugitech_Alim.pdf</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -737,54 +745,54 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>scanned</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>real_filled</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>JOB-2658</t>
+          <t>52498</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Suarez LLC Steel Mills</t>
+          <t>Ugitech SA</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Duplex 2205</t>
+          <t>Acier inoxydable / alliage</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>123.32 m</t>
+          <t>5 pages / 12+ nuances inox</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2025-10-12</t>
+          <t>2023-11-03</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Synthetic: Faker-generated data, complete ground truth.</t>
+          <t>Attestation d'alimentarité (food-grade) pour articles en acier inoxydable. Issued by Ugitech SA, Avenue Paul Girod, Ugine. Réf. Pdf 52498. Annexe lists 12+ EN-10088 grades (1.4301, 1.4307, 1.4401, 1.4404 etc.) compliant for food / drinking water contact across France, Belgique, USA.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Real_WeldingPlan_EN_Sandvik.pdf</t>
+          <t>Real_WeldingPlan_FR_Cahier_Soudage_Filtres.pdf</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -794,12 +802,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>scanned</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -809,45 +817,49 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>SS-011</t>
+          <t>00CD5528</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Sandvik</t>
+          <t>CFCE (manufacturer)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Hardox 450 / SS 2300 / SS2000 (50 &amp; 32 mm plates)</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+          <t>P355 NL1 / API 5L X52 (EN 10028-3)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>3 dampers (MAS-101 to MAS-104)</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2023-05-18</t>
+          <t>1998-04-21</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>WPS SS-011 rev 1.0, FCAW process. WPQR date 2023-03-07. Quantity N/A (procedure spec, not a material order).</t>
+          <t>Cahier de Soudage 'Filtres Séparateurs'. 24-page real welding dossier. Doc N° 5528-16-100 Rev.B. Customer IHI — 3 Discharge dampers 2nd stage. CFCE order 00CD5243. Fab N° 00-5243-104A/B/C. Norme CODAP95-ED.98/12 cat.B 1 + AM24.03.78. APAVE de l'Ouest inspections (VI/RS/RI 852EA 0007U) on 21/04/1998. WPS L1, C1, C2 referenced.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Real_WeldingPlan_EN_AWS_D17.1.pdf</t>
+          <t>Synthetic_MaterialCert_FR_01.pdf</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>WeldingPlan</t>
+          <t>MaterialCert</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -857,37 +869,49 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>real_template</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
+          <t>synthetic</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>PO-39290</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>AWS (D17.1/D17.1M:2010)</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
+          <t>Aubry Aciéries</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Monel 400</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>32.88 pcs</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2010-01-01</t>
+          <t>2024-01-13</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>AWS D17.1 WPS blank form template. All fillable fields empty. Date reflects standard edition, not a project.</t>
+          <t>Synthetic Faker-generated cert. Heat H-701949. Spec ASTM A580 / EN 10025. Inspector Louise Briand.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Real_WeldingPlan_FR_CEREMA_QMOS_DMOS.pdf</t>
+          <t>Synthetic_MaterialCert_FR_02.pdf</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>WeldingPlan</t>
+          <t>MaterialCert</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -902,25 +926,37 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>real_educational</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
+          <t>synthetic</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>PO-40824</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>CEREMA (Club Ouvrages d'Art Rhône-Alpes)</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
+          <t>Meyer Aciéries</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>SS 304</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>30.94 lbs</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2009-04-02</t>
+          <t>2025-09-02</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Educational presentation on QMOS/DMOS definitions (NF EN 15614-1, NF P 22 472). Author A. Houel, CETE de Lyon. No project-specific fields.</t>
+          <t>Synthetic Faker-generated cert. Heat H-929151. Spec ASTM A331 / EN 10025. Inspector William de la Boyer.</t>
         </is>
       </c>
     </row>
@@ -977,24 +1013,24 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Synthetic: Faker-generated data, complete ground truth.</t>
+          <t>Synthetic Faker-generated WPS. WPS-807-29. GTAW (TIG) procédé. Filler ER316L. Welder W-658.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Real_FabricationSheet_EN_DOE_Module2A.pdf</t>
+          <t>Synthetic_WeldingPlan_FR_02.pdf</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>FabricationSheet</t>
+          <t>WeldingPlan</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1004,28 +1040,44 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>real_educational</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
+          <t>synthetic</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>WO-22299</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>DOE (US Department of Energy)</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
+          <t>Marie</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Carbon Steel A36</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>456 units</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>2024-12-06</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Educational slide deck — 'Detailed Design Package Module 2A: Bill of Materials and Bill of Process'. No filled fields.</t>
+          <t>Synthetic Faker-generated WPS. WPS-901-62. SMAW procédé. Filler ER308L. Welder W-921. Approved by Martin Barbier du Bernard.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Real_FabricationSheet_FR_Goulet_Lecture_Plan_Soudage.pdf</t>
+          <t>Synthetic_FabricationSheet_FR_01.pdf</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1045,28 +1097,44 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>real_educational</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr"/>
+          <t>synthetic</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>PO-9326</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Goulet (textbook author)</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+          <t>Moulin</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Duplex 2205</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>149.58 lbs</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2024-09-14</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Textbook chapter 'Joints de base' — educational content about welding joint types. No project data.</t>
+          <t>Synthetic Faker-generated fiche de fabrication. Client Joly Gallet SA. Inspector Aurore Maury-Briand. Multi-line nomenclature.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_FabricationSheet_EN_01.pdf</t>
+          <t>Synthetic_FabricationSheet_FR_02.pdf</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1076,7 +1144,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1091,44 +1159,44 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>WLD-15592</t>
+          <t>WLD-67540</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Doyle Ltd</t>
+          <t>Gillet SA</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>SS 316</t>
+          <t>Copper C110</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>384 kg</t>
+          <t>106 lbs</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-01-24</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Synthetic: Faker-generated data, complete ground truth.</t>
+          <t>Synthetic Faker-generated fiche de fabrication. Client Barre. Inspector Julie Bertrand du Regnier. Multi-line nomenclature with 5 articles.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_FabricationSheet_FR_01.pdf</t>
+          <t>Synthetic_InspectionReport_FR_01.pdf</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>FabricationSheet</t>
+          <t>InspectionReport</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1148,39 +1216,39 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>PO-9326</t>
+          <t>PO-18172</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Moulin</t>
+          <t>Parent S.A.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Duplex 2205</t>
+          <t>Aluminium 6061-T6</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>149.58 lbs</t>
+          <t>220.39 pcs</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2024-09-14</t>
+          <t>2024-01-30</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Synthetic: Faker-generated data, complete ground truth.</t>
+          <t>Synthetic Faker-generated inspection report. IR-92578. Inspector Célina Colas. 4/5 contrôles CONFORME, étanchéité NON CONFORME.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Real_InspectionReport_EN_LANL_Weld.pdf</t>
+          <t>Synthetic_InspectionReport_FR_02.pdf</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1190,7 +1258,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1200,78 +1268,106 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>real_template</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr"/>
+          <t>synthetic</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>PRJ-30451</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>LANL (Los Alamos National Lab)</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
+          <t>Albert</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>SS 304</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>241 tons</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2006-10-27</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Weld Inspection Report form GWS 1-02-A3 Rev 1. Blank template — every field (Project/Code/Work Order/Base Material/Heat/Welder) unfilled.</t>
+          <t>Synthetic Faker-generated inspection report. IR-48254. Inspector Arnaude Petit. Mixed CONFORME / NON CONFORME results. Approved by Bernard Bernier.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Real_InspectionReport_EN_Trinity_VT_Report.pdf</t>
+          <t>Synthetic_Invoice_FR_01.pdf</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>InspectionReport</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>scanned</t>
+          <t>digital</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>real_template</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr"/>
+          <t>synthetic</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>FAB-71545</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Trinity NDT WeldSolutions Pvt. Ltd.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
+          <t>Moreau SARL</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Monel 400</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>381 tons</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>2024-08-12</t>
+        </is>
+      </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Weld Visual Testing (VT) report format TNE-VIR-05 Rev 0. Blank template. Vendor: Trinity NDT Bangalore India.</t>
+          <t>Synthetic Faker-generated facture. INV-45774. Client Étienne SARL. 4 line items. Total TTC 46293.26 €. Échéance 22/03/2025.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Real_InspectionReport_FR_Ifsttar_Auscultation.pdf</t>
+          <t>Synthetic_Invoice_FR_02.pdf</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>InspectionReport</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1286,47 +1382,59 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>real_educational</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr"/>
+          <t>synthetic</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>WLD-4552</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Ifsttar</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
+          <t>Leconte SARL</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>SS 304</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>108.01 kg</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2020-05-01</t>
+          <t>2024-02-21</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Collections Ifsttar Mai 2020 — guide 'Méthodes d'auscultation du matériau en place: acier / contrôle visuel et dimensionnel des soudures'. Educational, no project data.</t>
+          <t>Synthetic Faker-generated facture. INV-44099. Client Navarro. 4 line items. Total TTC 39515.34 €. Échéance 23/01/2025.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_InspectionReport_EN_01.pdf</t>
+          <t>Synthetic_MaterialCert_FR_01_scanned.pdf</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>InspectionReport</t>
+          <t>MaterialCert</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>scanned</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1336,85 +1444,101 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>WLD-43247</t>
+          <t>PO-39290</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Davis Group</t>
+          <t>Aubry Aciéries</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Copper C110</t>
+          <t>Monel 400</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>133 units</t>
+          <t>32.88 pcs</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2025-08-12</t>
+          <t>2024-01-13</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Synthetic: Faker-generated data, complete ground truth.</t>
+          <t>Scanned-modality variant of Synthetic_MaterialCert_FR_01 (degraded for OCR testing). Same Faker seed: Heat H-701949. Spec ASTM A580 / EN 10025. Inspector Louise Briand.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Real_Invoice_EN_Tennant.pdf</t>
+          <t>Synthetic_WeldingPlan_FR_01_scanned.pdf</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>WeldingPlan</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>scanned</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>real_template</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr"/>
+          <t>synthetic</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>WO-98154</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Tennant</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
+          <t>Bazin et Fils</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>PVC Sch 80</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>287 pcs</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>2024-03-18</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Commercial Invoice template (Tennant material#/description form). All 23 fields blank. Sample file '11.2 Sample Commercial Invoice.xls' export.</t>
+          <t>Scanned-modality variant of Synthetic_WeldingPlan_FR_01. Same Faker seed: WPS-807-29. GTAW (TIG). Filler ER316L. Welder W-658.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Real_Invoice_FR_Noyon.pdf</t>
+          <t>Synthetic_InspectionReport_FR_01_scanned.pdf</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>InspectionReport</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1424,33 +1548,49 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>scanned</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>real_template</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr"/>
+          <t>synthetic</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>PO-18172</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Noyon / P. Naggiar (consultant)</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
+          <t>Parent S.A.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Aluminium 6061-T6</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>220.39 pcs</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>2024-01-30</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Modèle de facture commerciale ou proforma (bilingual FR/EN). All fields blank.</t>
+          <t>Scanned-modality variant of Synthetic_InspectionReport_FR_01. Same Faker seed: IR-92578. Inspector Célina Colas.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_Invoice_EN_01.pdf</t>
+          <t>Synthetic_Invoice_FR_01_scanned.pdf</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1460,12 +1600,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>scanned</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1475,32 +1615,32 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>PO-1053</t>
+          <t>FAB-71545</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Harris, Collins and Carney Ltd.</t>
+          <t>Moreau SARL</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Aluminium 6061-T6</t>
+          <t>Monel 400</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>53.73 tons</t>
+          <t>381 tons</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>2025-03-28</t>
+          <t>2024-08-12</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Synthetic: Faker-generated data, complete ground truth.</t>
+          <t>Scanned-modality variant of Synthetic_Invoice_FR_01. Same Faker seed: INV-45774. Client Étienne SARL. Total TTC 46293.26 €.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pivot to French invoice scope (Tasks 1-5)
Old scope (5 doc types, 10 entities, EN+FR+synthetic) removed in full.
New scope: French invoices only, 11 entities including Solde du.

Tasks 1-5 delivered:
- Task 1: 19 unique French invoices organized in data/raw/french_invoices/
  (gitignored real client files; MANIFEST.md catalogs them)
- Task 2: docs/ground_truth.csv + .xlsx with 11 fields x 19 rows + Notes
- Task 3: docs/entity_schema.md with full French synonym matrix and
  accent-tolerance rules for every field
- Task 4: README rewritten; repo structure simplified to data/, docs/,
  scripts/, src/, tests/, outputs/extracted/
- Task 5: requirements.txt aligned with French OCR stack; setup notes
  for Tesseract fra pack documented in README

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ground_truth.xlsx
+++ b/docs/ground_truth.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ground Truth" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ground Truth'!$A$1:$K$21</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -42,7 +40,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,7 +58,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -431,1221 +428,1229 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>document_name</t>
+          <t>File Name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>doc_type</t>
+          <t>Supplier Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>language</t>
+          <t>Invoice Number</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>modality</t>
+          <t>Invoice Date</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>SIRET</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>project_id</t>
+          <t>Echeance</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>supplier</t>
+          <t>Invoice Content</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>material</t>
+          <t>TVA Percentage</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>TVA Amount</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>Total Amount</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>Payment Status</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Solde du</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Real_MaterialCert_FR_Larobinetterie_134822.pdf</t>
+          <t>IMG-20260507-WA0143.jpg</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MaterialCert</t>
+          <t>AOYAMA</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>T109200</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>real_filled</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>134822</t>
-        </is>
-      </c>
+          <t>44418819700016</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>La Robinetterie (LRI-Sodime)</t>
+          <t>1 Repas complet</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>1.4307 / 304L</t>
+          <t>10%; 20%</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>38 mm (dimension)</t>
+          <t>3,40 EUR</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2019-05-23</t>
+          <t>33,90 EUR</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Certificat de Réception 3.1 NF EN 10204. Heat number A1804323. Article 8185X.38 (TE SMS 38 INOX 304L).</t>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Justificatif de paiement; CB 33,90 EUR</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Real_MaterialCert_FR_Antelis_Dillinger_32.pdf</t>
+          <t>IMG-20260507-WA0144.jpg</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>MaterialCert</t>
+          <t>Hyper Carrefour Chalon</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>00031 00 02 00550383</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>real_filled</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>59003730</t>
-        </is>
-      </c>
+          <t>99269214500012</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>AG der Dillinger Hüttenwerke</t>
+          <t>Gazole 24,03 L @ 2,279 EUR/L</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>S355G10+N</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>15642 KG</t>
+          <t>9,13 EUR</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2018-09-26</t>
+          <t>54,76 EUR</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Certificat de Réception 3.2 EN 10204:2004. Customer: Antelis Leudelange. Heat 460073. Effective mass 15940 KG.</t>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Carte bancaire Visa - debit</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Real_MaterialCert_FR_Larobinetterie_160629.pdf</t>
+          <t>IMG-20260507-WA0145.jpg</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>MaterialCert</t>
+          <t>Orano Le Prisme</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>002-001-305604</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>real_filled</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>736145</t>
-        </is>
-      </c>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>SIDERINOX</t>
+          <t>Petit pain individuel; Conte AOP; Beurre portion x2; Eminence de boeuf</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>AISI 304/304L (EN 1.4301/1.4307)</t>
+          <t>10%; 20%</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>312 m</t>
+          <t>1,07 EUR</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2024-06-26</t>
+          <t>12,84 EUR</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Certificat d'essai EN 10204 3.1. Tube rond inox Ø 40 x 1 mm recuit brossé EN 10357 TC2 soudé. Client: La Robinetterie Industrielle. 284 kg poids total. DDT N°2725 du 26.06.2024.</t>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Cantine - badge interne; 'Solde 10,19' = solde du badge, pas de la facture</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Real_MaterialCert_FR_Dillinger_Antelis.pdf</t>
+          <t>IMG-20260507-WA0146.jpg</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>MaterialCert</t>
+          <t>Le Creusot Gare TGV (Effia)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>25557</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>real_filled</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>409707-001</t>
-        </is>
-      </c>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>AG der Dillinger Hüttenwerke</t>
+          <t>Stationnement Tarif 5 (Entree 17:31 / Paiement 22:31)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>S355K2+N</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>25434 KG</t>
+          <t>0,73 EUR</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2015-11-26</t>
+          <t>4,40 EUR</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Certificat de Réception 3.1 EN 10204:2004 / ISO 10474:2013. Customer: Antelis Leudelange. Avis d'expédition 6048684. 9 tôles 20x3000x6000 mm. Heat 427181. Norme NF-EN10025-2:05.</t>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Visa sans contact</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Real_MaterialCert_FR_Ugitech_Alim.pdf</t>
+          <t>IMG-20260507-WA0147.jpg</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>MaterialCert</t>
+          <t>La Boucherie Restaurant</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>134788</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>scanned</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>real_filled</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>52498</t>
-        </is>
-      </c>
+          <t>85214583800029</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Ugitech SA</t>
+          <t>1664 33CL; Tresor Louchebem; Garniture supplement; Supp sauce</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Acier inoxydable / alliage</t>
+          <t>10%; 20%</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>5 pages / 12+ nuances inox</t>
+          <t>4,39 EUR</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2023-11-03</t>
+          <t>43,50 EUR</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Attestation d'alimentarité (food-grade) pour articles en acier inoxydable. Issued by Ugitech SA, Avenue Paul Girod, Ugine. Réf. Pdf 52498. Annexe lists 12+ EN-10088 grades (1.4301, 1.4307, 1.4401, 1.4404 etc.) compliant for food / drinking water contact across France, Belgique, USA.</t>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>CB sans contact</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Real_WeldingPlan_FR_Cahier_Soudage_Filtres.pdf</t>
+          <t>IMG-20260507-WA0148.jpg</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>WeldingPlan</t>
+          <t>Studio Photo Lumiere &amp; Art</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>SPL-2024-0198</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>scanned</t>
+          <t>19/04/2024</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>real_filled</t>
+          <t>77789012300234</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>00CD5528</t>
+          <t>04/05/2024</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>CFCE (manufacturer)</t>
+          <t>Seance photo mariage (4h); Retouches numeriques (x80); Album photo 30x30 cm</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>P355 NL1 / API 5L X52 (EN 10028-3)</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>3 dampers (MAS-101 to MAS-104)</t>
+          <t>270,00 EUR</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>1998-04-21</t>
+          <t>1 620,00 EUR</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Cahier de Soudage 'Filtres Séparateurs'. 24-page real welding dossier. Doc N° 5528-16-100 Rev.B. Customer IHI — 3 Discharge dampers 2nd stage. CFCE order 00CD5243. Fab N° 00-5243-104A/B/C. Norme CODAP95-ED.98/12 cat.B 1 + AM24.03.78. APAVE de l'Ouest inspections (VI/RS/RI 852EA 0007U) on 21/04/1998. WPS L1, C1, C2 referenced.</t>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Conditions de reglement: Virement bancaire sous 15 jours</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_MaterialCert_FR_01.pdf</t>
+          <t>IMG-20260507-WA0149.jpg</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>MaterialCert</t>
+          <t>Clinique Dentaire Sourire</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CDS-2024-0345</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>16/04/2024</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>44456789100223</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>PO-39290</t>
+          <t>01/05/2024</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Aubry Aciéries</t>
+          <t>Detartrage complet; Soin carie molaire; Radiographie panoramique</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Monel 400</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>32.88 pcs</t>
+          <t>59,00 EUR</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2024-01-13</t>
+          <t>354,00 EUR</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Synthetic Faker-generated cert. Heat H-701949. Spec ASTM A580 / EN 10025. Inspector Louise Briand.</t>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Paye par Carte Bleue **** 2231 le 16/04/2024</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_MaterialCert_FR_02.pdf</t>
+          <t>IMG-20260507-WA0150.jpg</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>MaterialCert</t>
+          <t>Chauffage &amp; Climatisation Roux</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CCR-2024-0423</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>25/04/2024</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>99956789200267</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>PO-40824</t>
+          <t>25/05/2024</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Meyer Aciéries</t>
+          <t>Installation climatisation reversible; Mise en service et reglages; Garantie extension 3 ans</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>SS 304</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>30.94 lbs</t>
+          <t>225,00 EUR</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2025-09-02</t>
+          <t>2 475,00 EUR</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Synthetic Faker-generated cert. Heat H-929151. Spec ASTM A331 / EN 10025. Inspector William de la Boyer.</t>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Conditions: 40% commande, 60% reception - Virement ou cheque</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_WeldingPlan_FR_01.pdf</t>
+          <t>IMG-20260507-WA0151.jpg</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>WeldingPlan</t>
+          <t>Fleuriste Jardin d'Eden</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>FJE-2024-0087</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>23/04/2024</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>66623456700256</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>WO-98154</t>
+          <t>08/05/2024</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Bazin et Fils</t>
+          <t>Bouquet mariee rose &amp; pivoine; Decoration florale tables (x8); Composition entree salle</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>PVC Sch 80</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>287 pcs</t>
+          <t>82,00 EUR</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2024-03-18</t>
+          <t>902,00 EUR</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Synthetic Faker-generated WPS. WPS-807-29. GTAW (TIG) procédé. Filler ER316L. Welder W-658.</t>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Solde paye par American Express **** 8872 le 23/04/2024</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_WeldingPlan_FR_02.pdf</t>
+          <t>IMG-20260507-WA0152.jpg + IMG-20260507-WA0157.jpg</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>WeldingPlan</t>
+          <t>(non lisible - facture SCA010)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>FC20251175</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>synthetic</t>
-        </is>
-      </c>
+          <t>28/04/2025</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>WO-22299</t>
+          <t>28/05/2025</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Marie</t>
+          <t>AUDIT INITIAL ISO 19443 Etape 1 &amp; Etape 2; Certification ISO 9001 version 2015</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Carbon Steel A36</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>456 units</t>
+          <t>672,41 EUR</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>2024-12-06</t>
+          <t>4 034,46 EUR</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Synthetic Faker-generated WPS. WPS-901-62. SMAW procédé. Filler ER308L. Welder W-921. Approved by Martin Barbier du Bernard.</t>
+          <t>UNPAID</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>4 034,46 EUR</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Mode VIREMENT 30j net; N TVA intracom FR33845175751; deux photos = meme facture</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_FabricationSheet_FR_01.pdf</t>
+          <t>IMG-20260507-WA0153.jpg</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>FabricationSheet</t>
+          <t>Informatique Solutions Pro</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>ISP-2024-0512</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>21/04/2024</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>33390123400245</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>PO-9326</t>
+          <t>21/05/2024</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Moulin</t>
+          <t>Remplacement disque SSD 1To; Reinstallation Windows 11; Sauvegarde donnees (2h); Antivirus licence 1 an</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Duplex 2205</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>149.58 lbs</t>
+          <t>78,80 EUR</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2024-09-14</t>
+          <t>472,80 EUR</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Synthetic Faker-generated fiche de fabrication. Client Joly Gallet SA. Inspector Aurore Maury-Briand. Multi-line nomenclature.</t>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Paye par Visa **** 4491 le 22/04/2024</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_FabricationSheet_FR_02.pdf</t>
+          <t>IMG-20260507-WA0154.jpg + IMG-20260507-WA0158.jpg</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>FabricationSheet</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>digital</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>synthetic</t>
-        </is>
-      </c>
+          <t>(non lisible - fournisseur SCAI Systems)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>WLD-67540</t>
+          <t>15/11/2025</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Gillet SA</t>
+          <t>Scie radiale 1800W D355MM MKAS35 +2 lames; Lame scie D355x25,4x2,2mm 66 dts acier (x9); Lame scie supplementaire (x1)</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Copper C110</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>106 lbs</t>
+          <t>419,80 EUR</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2 518,81 EUR</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Synthetic Faker-generated fiche de fabrication. Client Barre. Inspector Julie Bertrand du Regnier. Multi-line nomenclature with 5 articles.</t>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Facture multi-pages; Mode Virement; Cde 08/09/2025; livre a SCAI Systems Le Creusot</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_InspectionReport_FR_01.pdf</t>
+          <t>IMG-20260507-WA0155.jpg</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>InspectionReport</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>digital</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>synthetic</t>
-        </is>
-      </c>
+          <t>Fers et Metaux du Chalonnais</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>PO-18172</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Parent S.A.</t>
+          <t>Corniere S235 JR 120x120x12; Poutrelle S275 JR IPE 270; Rond serrurier S235 JR Diam18; Corniere 25x25x3; TAC tole a chaud 1000x2000x15; Poutrelle UPN 100; Transport; Corniere 80x80x8</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Aluminium 6061-T6</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>220.39 pcs</t>
+          <t>1 309,13 EUR</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2024-01-30</t>
+          <t>7 854,77 EUR</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Synthetic Faker-generated inspection report. IR-92578. Inspector Célina Colas. 4/5 contrôles CONFORME, étanchéité NON CONFORME.</t>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Conditions de reglement: le 31/03/26; Acompte 0,00; Net a payer 7 854,77; Virement</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_InspectionReport_FR_02.pdf</t>
+          <t>IMG-20260507-WA0156.jpg</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>InspectionReport</t>
+          <t>Wurth Proxi Shop Le Creusot</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>digital</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>synthetic</t>
-        </is>
-      </c>
+          <t>4330739666</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>PRJ-30451</t>
+          <t>25/12/2024</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Albert</t>
+          <t>Disques a meuler MEULE EBARBER ZIRCO+ 230x6.4x22.2; Niveau digital IP65 61CM Zebra; Briquet USB electrique (offert); Coupon cadeau</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>SS 304</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>241 tons</t>
+          <t>136,50 EUR</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>818,98 EUR</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Synthetic Faker-generated inspection report. IR-48254. Inspector Arnaude Petit. Mixed CONFORME / NON CONFORME results. Approved by Bernard Bernier.</t>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Page 2/3 seulement; Conditions 30 jours; Mode Traite directe / Virement</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_Invoice_FR_01.pdf</t>
+          <t>Invoice_FR_016_scanned_260508_103316.pdf</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Epicerie Fine Marchand</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>EFM-2023-0412</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>12/11/2023</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>12378945600178</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>FAB-71545</t>
+          <t>27/11/2023</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Moreau SARL</t>
+          <t>Foie gras mi-cuit (4 boites) x6; Confiture artisanale (x12) x12; Huile d'olive AOC (4 flacons) x4</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Monel 400</t>
+          <t>5,5%</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>381 tons</t>
+          <t>19,24 EUR</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2024-08-12</t>
+          <t>369,04 EUR</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Synthetic Faker-generated facture. INV-45774. Client Étienne SARL. 4 line items. Total TTC 46293.26 €. Échéance 22/03/2025.</t>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Paye par Visa **** 4712 le 13/11/2023</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_Invoice_FR_02.pdf</t>
+          <t>Invoice_FR_017_scanned_260508_103241.pdf</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Atelier Couture &amp; Retouches Blondel</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>ACR-2023-1205</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>05/12/2023</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>55534567900169</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>WLD-4552</t>
+          <t>20/12/2023</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Leconte SARL</t>
+          <t>Retouche robe de mariee; Ourlet pantalon (x3); Remplacement fermeture eclair</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>SS 304</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>108.01 kg</t>
+          <t>50,00 EUR</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2024-02-21</t>
+          <t>300,00 EUR</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Synthetic Faker-generated facture. INV-44099. Client Navarro. 4 line items. Total TTC 39515.34 €. Échéance 23/01/2025.</t>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Especes recues - recu N 2023-1205</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_MaterialCert_FR_01_scanned.pdf</t>
+          <t>Invoice_FR_018_scanned_260508_103257.pdf</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>MaterialCert</t>
+          <t>Garage Mecanique Verdier</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>GMV-2023-0789</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>scanned</t>
+          <t>28/10/2023</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>88801234600190</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>PO-39290</t>
+          <t>12/11/2023</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Aubry Aciéries</t>
+          <t>Vidange + filtre huile; Remplacement plaquettes frein AV; Main d'oeuvre revision (3h); Pneumatiques 195/65 R15 (x2)</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Monel 400</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>32.88 pcs</t>
+          <t>121,20 EUR</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2024-01-13</t>
+          <t>727,20 EUR</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Scanned-modality variant of Synthetic_MaterialCert_FR_01 (degraded for OCR testing). Same Faker seed: Heat H-701949. Spec ASTM A580 / EN 10025. Inspector Louise Briand.</t>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Conditions de reglement: Cheque a l'ordre de Garage Verdier sous 15 jours</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_WeldingPlan_FR_01_scanned.pdf</t>
+          <t>Invoice_FR_019_scanned_260508_103345.pdf</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>WeldingPlan</t>
+          <t>Ecole de Musique Harmonie</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>EMH-2024-0023</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>scanned</t>
+          <t>08/01/2024</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>33345678900201</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>WO-98154</t>
+          <t>08/02/2024</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Bazin et Fils</t>
+          <t>Cours de piano - trimestre 1 (x12 seances); Location salle de repetition (x4h); Partition recueil Bach</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>PVC Sch 80</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>287 pcs</t>
+          <t>127,70 EUR</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>2024-03-18</t>
+          <t>766,20 EUR</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Scanned-modality variant of Synthetic_WeldingPlan_FR_01. Same Faker seed: WPS-807-29. GTAW (TIG). Filler ER316L. Welder W-658.</t>
+          <t>PAID</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Reglement par CB Mastercard **** 3308 accepte le 09/01/2024</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Synthetic_InspectionReport_FR_01_scanned.pdf</t>
+          <t>Invoice_FR_020_scanned_260508_103334.pdf</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>InspectionReport</t>
+          <t>Paysagiste Terrain Vert EURL</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>PTV-2024-0156</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>scanned</t>
+          <t>22/02/2024</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>66612890100212</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>PO-18172</t>
+          <t>08/03/2024</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Parent S.A.</t>
+          <t>Tonte pelouse + ramassage (x4 passages); Taille haies et arbustes; Plantation massif fleuri (x15 plants); Evacuation dechets verts</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Aluminium 6061-T6</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>220.39 pcs</t>
+          <t>73,50 EUR</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>2024-01-30</t>
+          <t>808,50 EUR</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Scanned-modality variant of Synthetic_InspectionReport_FR_01. Same Faker seed: IR-92578. Inspector Célina Colas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Synthetic_Invoice_FR_01_scanned.pdf</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>scanned</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>synthetic</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>FAB-71545</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>Moreau SARL</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Monel 400</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>381 tons</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>2024-08-12</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Scanned-modality variant of Synthetic_Invoice_FR_01. Same Faker seed: INV-45774. Client Étienne SARL. Total TTC 46293.26 €.</t>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Conditions de reglement: Virement IBAN FR76 3000 6228 3700 0100 0000 - a regler avant le 08/03/2024</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>